<commit_message>
Final commit, documentation added: -report -assessment -query example
</commit_message>
<xml_diff>
--- a/MainDirectory/report/Self Assessment Form - IUM-TWEB.xlsx
+++ b/MainDirectory/report/Self Assessment Form - IUM-TWEB.xlsx
@@ -980,7 +980,7 @@
         <v>24</v>
       </c>
       <c r="D23" s="18">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1">
@@ -998,7 +998,7 @@
         <v>26</v>
       </c>
       <c r="D25" s="18">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="26" ht="16.5" customHeight="1">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="C53" s="13"/>
       <c r="D53" s="18">
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="54" ht="16.5" customHeight="1">

</xml_diff>